<commit_message>
Separate Detachment and School markers into their own components
</commit_message>
<xml_diff>
--- a/Schools.xlsx
+++ b/Schools.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sgreenwood/Projects/work/recruitment-area.acf.university-projects.com/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D136DD1E-A275-4542-8E30-35A946679A7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07E47939-E3AE-4041-B431-7FAD16EF7FF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3080" yWindow="2160" windowWidth="28040" windowHeight="17180" xr2:uid="{2A2DEAA7-4276-AE4C-A0FC-71E357318295}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="72">
   <si>
     <t>Area</t>
   </si>
@@ -252,6 +252,9 @@
   </si>
   <si>
     <t>Broadway, Fleetwood, FY7 8JW</t>
+  </si>
+  <si>
+    <t>Added</t>
   </si>
 </sst>
 </file>
@@ -287,13 +290,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -306,10 +324,32 @@
 </styleSheet>
 </file>
 
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+  <bag type="DXFComplements" extRef="DXFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C2F0B9CE-5036-C046-AC39-9524D6736052}" name="Table2" displayName="Table2" ref="A1:G30" totalsRowShown="0">
-  <autoFilter ref="A1:G30" xr:uid="{C2F0B9CE-5036-C046-AC39-9524D6736052}"/>
-  <tableColumns count="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C2F0B9CE-5036-C046-AC39-9524D6736052}" name="Table2" displayName="Table2" ref="A1:H30" totalsRowShown="0">
+  <autoFilter ref="A1:H30" xr:uid="{C2F0B9CE-5036-C046-AC39-9524D6736052}"/>
+  <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{1A5ADD18-5E4C-DC46-9EEC-91A6915593D0}" name="Area"/>
     <tableColumn id="2" xr3:uid="{2E6AB0B7-E731-E342-B53C-4E0D9CED348F}" name="Name"/>
     <tableColumn id="3" xr3:uid="{02517E76-DDCC-4D41-8AE9-98B76F192E3A}" name="Address"/>
@@ -317,6 +357,7 @@
     <tableColumn id="5" xr3:uid="{0D91B1A7-E362-664B-9EF2-F6EFE15E3373}" name="Longitude"/>
     <tableColumn id="6" xr3:uid="{CBD550C9-21BA-0D47-BBBE-C2FAFA6A7635}" name="State/Private"/>
     <tableColumn id="7" xr3:uid="{29C02D26-7915-0D4C-87E5-607FC1299D55}" name="Estimated number of pupils"/>
+    <tableColumn id="8" xr3:uid="{F9322AE1-936F-6D48-9CFA-4DE878CFD76E}" name="Added" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -639,7 +680,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{664134CA-CB6B-0D44-9BED-5E1A97F81731}">
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.1640625" bestFit="1" customWidth="1"/>
@@ -651,7 +692,7 @@
     <col min="7" max="7" width="26.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -673,8 +714,11 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -696,8 +740,11 @@
       <c r="G2">
         <v>1221</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H2" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -719,8 +766,11 @@
       <c r="G3">
         <v>799</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H3" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -742,8 +792,11 @@
       <c r="G4">
         <v>751</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H4" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -765,8 +818,11 @@
       <c r="G5">
         <v>1192</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H5" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -788,8 +844,11 @@
       <c r="G6">
         <v>550</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H6" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -811,8 +870,11 @@
       <c r="G7">
         <v>609</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H7" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -834,8 +896,11 @@
       <c r="G8">
         <v>1188</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H8" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -857,8 +922,11 @@
       <c r="G9">
         <v>877</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H9" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -880,8 +948,11 @@
       <c r="G10">
         <v>790</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H10" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -903,8 +974,11 @@
       <c r="G11">
         <v>1588</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H11" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -926,8 +1000,11 @@
       <c r="G12">
         <v>831</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H12" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -949,8 +1026,11 @@
       <c r="G13">
         <v>785</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H13" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>25</v>
       </c>
@@ -972,8 +1052,11 @@
       <c r="G14">
         <v>670</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H14" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>37</v>
       </c>
@@ -995,8 +1078,11 @@
       <c r="G15">
         <v>724</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H15" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>37</v>
       </c>
@@ -1018,8 +1104,11 @@
       <c r="G16">
         <v>657</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H16" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>37</v>
       </c>
@@ -1041,8 +1130,11 @@
       <c r="G17">
         <v>1038</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H17" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>37</v>
       </c>
@@ -1064,8 +1156,11 @@
       <c r="G18">
         <v>567</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H18" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -1087,8 +1182,11 @@
       <c r="G19">
         <v>1294</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H19" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>37</v>
       </c>
@@ -1110,8 +1208,11 @@
       <c r="G20">
         <v>1045</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H20" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>37</v>
       </c>
@@ -1133,8 +1234,11 @@
       <c r="G21">
         <v>981</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H21" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>37</v>
       </c>
@@ -1156,8 +1260,11 @@
       <c r="G22">
         <v>1755</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H22" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>54</v>
       </c>
@@ -1179,8 +1286,11 @@
       <c r="G23">
         <v>726</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H23" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>54</v>
       </c>
@@ -1202,8 +1312,11 @@
       <c r="G24">
         <v>769</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H24" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>54</v>
       </c>
@@ -1225,8 +1338,11 @@
       <c r="G25">
         <v>1025</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H25" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>54</v>
       </c>
@@ -1248,8 +1364,11 @@
       <c r="G26">
         <v>750</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H26" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>54</v>
       </c>
@@ -1271,8 +1390,11 @@
       <c r="G27">
         <v>1121</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H27" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>54</v>
       </c>
@@ -1294,8 +1416,11 @@
       <c r="G28">
         <v>873</v>
       </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H28" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>54</v>
       </c>
@@ -1317,8 +1442,11 @@
       <c r="G29">
         <v>820</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H29" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>54</v>
       </c>
@@ -1340,9 +1468,13 @@
       <c r="G30">
         <v>810</v>
       </c>
+      <c r="H30" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>